<commit_message>
best conclusions with strength of alignment
</commit_message>
<xml_diff>
--- a/OUTPUT_REPORT/best_conclusion_data.xlsx
+++ b/OUTPUT_REPORT/best_conclusion_data.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drippy/OUTPUT_REPORT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{374ECCFF-6BB2-7546-9D31-4ECC5D5735DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C02FF9-78AB-B247-A6CB-6E241CB21F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="7580" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$69</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="543">
   <si>
     <t>Family</t>
   </si>
@@ -76,7 +79,7 @@
     <t>Inverted_Pval</t>
   </si>
   <si>
-    <t>Disagreement</t>
+    <t>Alignment</t>
   </si>
   <si>
     <t>LexA</t>
@@ -115,6 +118,9 @@
     <t>GAA</t>
   </si>
   <si>
+    <t>Weak agree</t>
+  </si>
+  <si>
     <t>Q9ZFA4</t>
   </si>
   <si>
@@ -196,6 +202,9 @@
     <t>GTTC</t>
   </si>
   <si>
+    <t>Strong agree</t>
+  </si>
+  <si>
     <t>Bdellovibrio_bacteriovorus_HD100</t>
   </si>
   <si>
@@ -283,6 +292,9 @@
     <t>TAA</t>
   </si>
   <si>
+    <t>Strong disagree</t>
+  </si>
+  <si>
     <t>Q9A724</t>
   </si>
   <si>
@@ -635,6 +647,9 @@
   </si>
   <si>
     <t>CA</t>
+  </si>
+  <si>
+    <t>Weak disagree</t>
   </si>
   <si>
     <t>Geobacter_sulfurreducens_PCA</t>
@@ -1655,6 +1670,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1999,11 +2015,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:S69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="35.5" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -2066,58 +2080,61 @@
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="I2" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>85</v>
+      </c>
+      <c r="K2" t="s">
+        <v>86</v>
       </c>
       <c r="L2" t="s">
-        <v>29</v>
+        <v>87</v>
       </c>
       <c r="M2">
         <v>3</v>
       </c>
       <c r="N2">
-        <v>5.4229728339368526</v>
+        <v>4.3939234320752298</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="P2" t="s">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="Q2">
-        <v>8.0167932826869251E-2</v>
+        <v>2.0391843262694921E-2</v>
       </c>
       <c r="R2">
-        <v>0.91983206717313071</v>
-      </c>
-      <c r="S2" t="b">
-        <v>0</v>
+        <v>0.97960815673730506</v>
+      </c>
+      <c r="S2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
@@ -2125,55 +2142,52 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>107</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>108</v>
       </c>
       <c r="I3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="L3" t="s">
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N3">
-        <v>11.99999993760844</v>
+        <v>2.9773800562974402</v>
       </c>
       <c r="O3" t="s">
-        <v>37</v>
+        <v>111</v>
       </c>
       <c r="P3" t="s">
-        <v>37</v>
+        <v>111</v>
       </c>
       <c r="Q3">
-        <v>0.1105557776889244</v>
+        <v>2.2990803678528592E-2</v>
       </c>
       <c r="R3">
-        <v>0.88944422231107556</v>
-      </c>
-      <c r="S3" t="b">
-        <v>0</v>
+        <v>0.97700919632147143</v>
+      </c>
+      <c r="S3" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -2181,90 +2195,93 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>377</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>378</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>379</v>
       </c>
       <c r="H4" t="s">
-        <v>42</v>
+        <v>380</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>381</v>
       </c>
       <c r="J4" t="s">
-        <v>44</v>
+        <v>28</v>
+      </c>
+      <c r="K4" t="s">
+        <v>382</v>
       </c>
       <c r="L4" t="s">
-        <v>45</v>
+        <v>383</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4">
-        <v>9.9999999480070354</v>
+        <v>4.9999999694042216</v>
       </c>
       <c r="O4" t="s">
-        <v>46</v>
+        <v>384</v>
       </c>
       <c r="P4" t="s">
-        <v>46</v>
+        <v>385</v>
       </c>
       <c r="Q4">
-        <v>0.62714914034386249</v>
+        <v>2.119152339064374E-2</v>
       </c>
       <c r="R4">
-        <v>0.37285085965613751</v>
-      </c>
-      <c r="S4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.97880847660935622</v>
+      </c>
+      <c r="S4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M5">
         <v>4</v>
@@ -2273,10 +2290,10 @@
         <v>6.6208370719702616</v>
       </c>
       <c r="O5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q5">
         <v>1.9992003198720509E-4</v>
@@ -2284,8 +2301,8 @@
       <c r="R5">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S5" t="b">
-        <v>0</v>
+      <c r="S5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
@@ -2293,84 +2310,87 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>469</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>470</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>471</v>
       </c>
       <c r="G6" t="s">
-        <v>61</v>
+        <v>472</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>473</v>
       </c>
       <c r="I6" t="s">
-        <v>63</v>
+        <v>474</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
       </c>
       <c r="L6" t="s">
-        <v>64</v>
+        <v>475</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N6">
-        <v>7.9999999584056276</v>
+        <v>11.99999993760844</v>
       </c>
       <c r="O6" t="s">
-        <v>65</v>
+        <v>476</v>
       </c>
       <c r="P6" t="s">
-        <v>66</v>
+        <v>476</v>
       </c>
       <c r="Q6">
-        <v>5.9376249500199922E-2</v>
+        <v>3.7984806077568968E-3</v>
       </c>
       <c r="R6">
-        <v>0.94062375049980007</v>
-      </c>
-      <c r="S6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.99620151939224311</v>
+      </c>
+      <c r="S6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="M7">
         <v>4</v>
@@ -2379,10 +2399,10 @@
         <v>7.1887218374956996</v>
       </c>
       <c r="O7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="Q7">
         <v>7.9968012794882047E-4</v>
@@ -2390,78 +2410,72 @@
       <c r="R7">
         <v>0.99920031987205116</v>
       </c>
-      <c r="S7" t="b">
-        <v>0</v>
+      <c r="S7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>521</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>529</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>79</v>
+        <v>530</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
+        <v>531</v>
       </c>
       <c r="H8" t="s">
-        <v>81</v>
+        <v>532</v>
       </c>
       <c r="I8" t="s">
-        <v>82</v>
-      </c>
-      <c r="J8" t="s">
-        <v>83</v>
-      </c>
-      <c r="K8" t="s">
-        <v>84</v>
+        <v>533</v>
       </c>
       <c r="L8" t="s">
-        <v>85</v>
+        <v>534</v>
       </c>
       <c r="M8">
         <v>3</v>
       </c>
       <c r="N8">
-        <v>4.3939234320752298</v>
+        <v>3.2715463687802688</v>
       </c>
       <c r="O8" t="s">
-        <v>86</v>
+        <v>535</v>
       </c>
       <c r="P8" t="s">
-        <v>86</v>
+        <v>536</v>
       </c>
       <c r="Q8">
-        <v>2.0391843262694921E-2</v>
+        <v>1.9192323070771691E-2</v>
       </c>
       <c r="R8">
-        <v>0.97960815673730506</v>
-      </c>
-      <c r="S8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.98080767692922832</v>
+      </c>
+      <c r="S8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -2470,19 +2484,19 @@
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="L9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="M9">
         <v>5</v>
@@ -2491,10 +2505,10 @@
         <v>7.8883833705737496</v>
       </c>
       <c r="O9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="P9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q9">
         <v>1.9992003198720509E-4</v>
@@ -2502,19 +2516,19 @@
       <c r="R9">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
@@ -2523,22 +2537,22 @@
         <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H10" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I10" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="J10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L10" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M10">
         <v>4</v>
@@ -2547,10 +2561,10 @@
         <v>5.2998582469101541</v>
       </c>
       <c r="O10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="Q10">
         <v>1.9992003198720509E-4</v>
@@ -2558,8 +2572,8 @@
       <c r="R10">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S10" t="b">
-        <v>0</v>
+      <c r="S10" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
@@ -2567,137 +2581,143 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
         <v>23</v>
       </c>
       <c r="F11" t="s">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="I11" t="s">
-        <v>106</v>
+        <v>27</v>
+      </c>
+      <c r="J11" t="s">
+        <v>28</v>
       </c>
       <c r="L11" t="s">
-        <v>107</v>
+        <v>29</v>
       </c>
       <c r="M11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11">
-        <v>2.9773800562974402</v>
+        <v>5.4229728339368526</v>
       </c>
       <c r="O11" t="s">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="P11" t="s">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="Q11">
-        <v>2.2990803678528592E-2</v>
+        <v>8.0167932826869251E-2</v>
       </c>
       <c r="R11">
-        <v>0.97700919632147143</v>
-      </c>
-      <c r="S11" t="b">
-        <v>1</v>
+        <v>0.91983206717313071</v>
+      </c>
+      <c r="S11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J12" t="s">
+        <v>28</v>
+      </c>
+      <c r="L12" t="s">
+        <v>37</v>
+      </c>
+      <c r="M12">
+        <v>6</v>
+      </c>
+      <c r="N12">
+        <v>11.99999993760844</v>
+      </c>
+      <c r="O12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q12">
+        <v>0.1105557776889244</v>
+      </c>
+      <c r="R12">
+        <v>0.88944422231107556</v>
+      </c>
+      <c r="S12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s">
         <v>50</v>
       </c>
-      <c r="F12" t="s">
-        <v>111</v>
-      </c>
-      <c r="G12" t="s">
-        <v>112</v>
-      </c>
-      <c r="H12" t="s">
-        <v>113</v>
-      </c>
-      <c r="I12" t="s">
-        <v>114</v>
-      </c>
-      <c r="L12" t="s">
-        <v>115</v>
-      </c>
-      <c r="M12">
-        <v>3</v>
-      </c>
-      <c r="N12">
-        <v>4.2408072171713433</v>
-      </c>
-      <c r="O12" t="s">
-        <v>116</v>
-      </c>
-      <c r="P12" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q12">
-        <v>9.9160335865653745E-2</v>
-      </c>
-      <c r="R12">
-        <v>0.90083966413434624</v>
-      </c>
-      <c r="S12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B13" t="s">
-        <v>118</v>
-      </c>
-      <c r="C13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D13" t="s">
-        <v>49</v>
-      </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G13" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H13" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I13" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="L13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M13">
         <v>3</v>
@@ -2706,10 +2726,10 @@
         <v>4.3226574925258454</v>
       </c>
       <c r="O13" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P13" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q13">
         <v>7.9968012794882047E-4</v>
@@ -2717,43 +2737,43 @@
       <c r="R13">
         <v>0.99920031987205116</v>
       </c>
-      <c r="S13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G14" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H14" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="I14" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L14" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="M14">
         <v>6</v>
@@ -2762,10 +2782,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="P14" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="Q14">
         <v>5.9976009596161544E-3</v>
@@ -2773,43 +2793,43 @@
       <c r="R14">
         <v>0.9940023990403839</v>
       </c>
-      <c r="S14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G15" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H15" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I15" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="J15" t="s">
         <v>28</v>
       </c>
       <c r="L15" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="M15">
         <v>4</v>
@@ -2818,10 +2838,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O15" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="P15" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="Q15">
         <v>1.8192722910835669E-2</v>
@@ -2829,43 +2849,43 @@
       <c r="R15">
         <v>0.98180727708916438</v>
       </c>
-      <c r="S15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F16" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G16" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H16" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I16" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="J16" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="L16" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="M16">
         <v>6</v>
@@ -2874,10 +2894,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O16" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="P16" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="Q16">
         <v>3.9984006397441018E-4</v>
@@ -2885,43 +2905,43 @@
       <c r="R16">
         <v>0.99960015993602558</v>
       </c>
-      <c r="S16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C17" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F17" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="G17" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="H17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I17" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J17" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="L17" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="M17">
         <v>3</v>
@@ -2930,10 +2950,10 @@
         <v>5.3600982884038064</v>
       </c>
       <c r="O17" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="P17" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="Q17">
         <v>2.1991203518592559E-3</v>
@@ -2941,72 +2961,75 @@
       <c r="R17">
         <v>0.99780087964814079</v>
       </c>
-      <c r="S17" t="b">
-        <v>0</v>
+      <c r="S17" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>151</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>159</v>
+        <v>40</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F18" t="s">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="G18" t="s">
-        <v>161</v>
+        <v>42</v>
       </c>
       <c r="H18" t="s">
-        <v>162</v>
+        <v>43</v>
       </c>
       <c r="I18" t="s">
-        <v>163</v>
+        <v>44</v>
+      </c>
+      <c r="J18" t="s">
+        <v>45</v>
       </c>
       <c r="L18" t="s">
-        <v>164</v>
+        <v>46</v>
       </c>
       <c r="M18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N18">
-        <v>2.6564805730254588</v>
+        <v>9.9999999480070354</v>
       </c>
       <c r="O18" t="s">
-        <v>165</v>
+        <v>47</v>
       </c>
       <c r="P18" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="Q18">
-        <v>0.38604558176729309</v>
+        <v>0.62714914034386249</v>
       </c>
       <c r="R18">
-        <v>0.61395441823270691</v>
-      </c>
-      <c r="S18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.37285085965613751</v>
+      </c>
+      <c r="S18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -3015,19 +3038,19 @@
         <v>23</v>
       </c>
       <c r="F19" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G19" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H19" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="I19" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="L19" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="M19">
         <v>4</v>
@@ -3036,10 +3059,10 @@
         <v>5.2017458551690039</v>
       </c>
       <c r="O19" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="P19" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="Q19">
         <v>1.9992003198720509E-4</v>
@@ -3047,40 +3070,40 @@
       <c r="R19">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S19" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C20" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G20" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H20" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="I20" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="L20" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="M20">
         <v>4</v>
@@ -3089,10 +3112,10 @@
         <v>5.6466531753055396</v>
       </c>
       <c r="O20" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="P20" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Q20">
         <v>1.9992003198720509E-4</v>
@@ -3100,19 +3123,19 @@
       <c r="R20">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S20" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C21" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D21" t="s">
         <v>22</v>
@@ -3121,22 +3144,22 @@
         <v>23</v>
       </c>
       <c r="F21" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G21" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H21" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="I21" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="J21" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="L21" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="M21">
         <v>4</v>
@@ -3145,10 +3168,10 @@
         <v>4.274987873675073</v>
       </c>
       <c r="O21" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="P21" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="Q21">
         <v>2.1991203518592559E-3</v>
@@ -3156,19 +3179,19 @@
       <c r="R21">
         <v>0.99780087964814079</v>
       </c>
-      <c r="S21" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C22" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -3177,22 +3200,22 @@
         <v>23</v>
       </c>
       <c r="F22" t="s">
+        <v>193</v>
+      </c>
+      <c r="G22" t="s">
+        <v>194</v>
+      </c>
+      <c r="H22" t="s">
+        <v>195</v>
+      </c>
+      <c r="I22" t="s">
+        <v>196</v>
+      </c>
+      <c r="J22" t="s">
         <v>190</v>
       </c>
-      <c r="G22" t="s">
-        <v>191</v>
-      </c>
-      <c r="H22" t="s">
-        <v>192</v>
-      </c>
-      <c r="I22" t="s">
-        <v>193</v>
-      </c>
-      <c r="J22" t="s">
-        <v>187</v>
-      </c>
       <c r="L22" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="M22">
         <v>5</v>
@@ -3201,10 +3224,10 @@
         <v>7.6068990586698382</v>
       </c>
       <c r="O22" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="P22" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="Q22">
         <v>2.9988004798080772E-3</v>
@@ -3212,8 +3235,8 @@
       <c r="R22">
         <v>0.99700119952019195</v>
       </c>
-      <c r="S22" t="b">
-        <v>0</v>
+      <c r="S22" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
@@ -3221,143 +3244,137 @@
         <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>196</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>197</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F23" t="s">
-        <v>198</v>
+        <v>62</v>
       </c>
       <c r="G23" t="s">
-        <v>199</v>
+        <v>63</v>
       </c>
       <c r="H23" t="s">
-        <v>200</v>
+        <v>64</v>
       </c>
       <c r="I23" t="s">
-        <v>201</v>
-      </c>
-      <c r="J23" t="s">
-        <v>202</v>
+        <v>65</v>
       </c>
       <c r="L23" t="s">
-        <v>203</v>
+        <v>66</v>
       </c>
       <c r="M23">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N23">
-        <v>3.422972844335447</v>
+        <v>7.9999999584056276</v>
       </c>
       <c r="O23" t="s">
-        <v>204</v>
+        <v>67</v>
       </c>
       <c r="P23" t="s">
-        <v>204</v>
+        <v>68</v>
       </c>
       <c r="Q23">
-        <v>0.1239504198320672</v>
+        <v>5.9376249500199922E-2</v>
       </c>
       <c r="R23">
-        <v>0.87604958016793288</v>
-      </c>
-      <c r="S23" t="b">
-        <v>1</v>
+        <v>0.94062375049980007</v>
+      </c>
+      <c r="S23" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="B24" t="s">
-        <v>205</v>
+        <v>104</v>
       </c>
       <c r="C24" t="s">
-        <v>206</v>
+        <v>113</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F24" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="G24" t="s">
-        <v>208</v>
+        <v>115</v>
       </c>
       <c r="H24" t="s">
-        <v>209</v>
+        <v>116</v>
       </c>
       <c r="I24" t="s">
-        <v>210</v>
-      </c>
-      <c r="J24" t="s">
-        <v>28</v>
+        <v>117</v>
       </c>
       <c r="L24" t="s">
-        <v>211</v>
+        <v>118</v>
       </c>
       <c r="M24">
         <v>3</v>
       </c>
       <c r="N24">
-        <v>5.9999999688042216</v>
+        <v>4.2408072171713433</v>
       </c>
       <c r="O24" t="s">
-        <v>212</v>
+        <v>119</v>
       </c>
       <c r="P24" t="s">
-        <v>213</v>
+        <v>120</v>
       </c>
       <c r="Q24">
-        <v>0.2387045181927229</v>
+        <v>9.9160335865653745E-2</v>
       </c>
       <c r="R24">
-        <v>0.76129548180727713</v>
-      </c>
-      <c r="S24" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.90083966413434624</v>
+      </c>
+      <c r="S24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C25" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F25" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G25" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="H25" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="I25" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="L25" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="M25">
         <v>3</v>
@@ -3366,10 +3383,10 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O25" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="P25" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="Q25">
         <v>3.398640543782487E-3</v>
@@ -3377,40 +3394,40 @@
       <c r="R25">
         <v>0.99660135945621753</v>
       </c>
-      <c r="S25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S25" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C26" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F26" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="G26" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H26" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="I26" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="L26" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="M26">
         <v>3</v>
@@ -3419,10 +3436,10 @@
         <v>4.8459456990694862</v>
       </c>
       <c r="O26" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="P26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="Q26">
         <v>1.5993602558976409E-2</v>
@@ -3430,96 +3447,93 @@
       <c r="R26">
         <v>0.98400639744102358</v>
       </c>
-      <c r="S26" t="b">
-        <v>0</v>
+      <c r="S26" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="B27" t="s">
-        <v>230</v>
+        <v>154</v>
       </c>
       <c r="C27" t="s">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="D27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E27" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F27" t="s">
-        <v>232</v>
+        <v>163</v>
       </c>
       <c r="G27" t="s">
-        <v>233</v>
+        <v>164</v>
       </c>
       <c r="H27" t="s">
-        <v>234</v>
+        <v>165</v>
       </c>
       <c r="I27" t="s">
-        <v>235</v>
-      </c>
-      <c r="J27" t="s">
-        <v>44</v>
+        <v>166</v>
       </c>
       <c r="L27" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="M27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N27">
-        <v>7.9999999584056276</v>
+        <v>2.6564805730254588</v>
       </c>
       <c r="O27" t="s">
-        <v>237</v>
+        <v>168</v>
       </c>
       <c r="P27" t="s">
-        <v>238</v>
+        <v>169</v>
       </c>
       <c r="Q27">
-        <v>0.22491003598560569</v>
+        <v>0.38604558176729309</v>
       </c>
       <c r="R27">
-        <v>0.77508996401439423</v>
-      </c>
-      <c r="S27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.61395441823270691</v>
+      </c>
+      <c r="S27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>19</v>
       </c>
       <c r="B28" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C28" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F28" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="G28" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H28" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I28" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="L28" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="M28">
         <v>4</v>
@@ -3528,10 +3542,10 @@
         <v>6.4237692198623009</v>
       </c>
       <c r="O28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P28" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q28">
         <v>1.9992003198720509E-4</v>
@@ -3539,43 +3553,43 @@
       <c r="R28">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S28" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C29" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E29" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F29" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="G29" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="H29" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="I29" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="J29" t="s">
         <v>28</v>
       </c>
       <c r="L29" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="M29">
         <v>4</v>
@@ -3584,10 +3598,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O29" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="P29" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="Q29">
         <v>9.1963214714114363E-3</v>
@@ -3595,8 +3609,8 @@
       <c r="R29">
         <v>0.99080367852858853</v>
       </c>
-      <c r="S29" t="b">
-        <v>0</v>
+      <c r="S29" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
@@ -3604,90 +3618,90 @@
         <v>19</v>
       </c>
       <c r="B30" t="s">
-        <v>255</v>
+        <v>209</v>
       </c>
       <c r="C30" t="s">
-        <v>256</v>
+        <v>210</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E30" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F30" t="s">
-        <v>257</v>
+        <v>211</v>
       </c>
       <c r="G30" t="s">
-        <v>258</v>
+        <v>212</v>
       </c>
       <c r="H30" t="s">
-        <v>259</v>
+        <v>213</v>
       </c>
       <c r="I30" t="s">
-        <v>260</v>
+        <v>214</v>
       </c>
       <c r="J30" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="L30" t="s">
-        <v>261</v>
+        <v>215</v>
       </c>
       <c r="M30">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N30">
-        <v>7.9999999584056276</v>
+        <v>5.9999999688042216</v>
       </c>
       <c r="O30" t="s">
-        <v>139</v>
+        <v>216</v>
       </c>
       <c r="P30" t="s">
-        <v>140</v>
+        <v>217</v>
       </c>
       <c r="Q30">
-        <v>0.1273490603758497</v>
+        <v>0.2387045181927229</v>
       </c>
       <c r="R30">
-        <v>0.8726509396241503</v>
-      </c>
-      <c r="S30" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.76129548180727713</v>
+      </c>
+      <c r="S30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>19</v>
       </c>
       <c r="B31" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C31" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F31" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="G31" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="H31" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="I31" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L31" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="M31">
         <v>5</v>
@@ -3696,10 +3710,10 @@
         <v>9.9999999480070354</v>
       </c>
       <c r="O31" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="P31" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q31">
         <v>6.9972011195521804E-3</v>
@@ -3707,43 +3721,43 @@
       <c r="R31">
         <v>0.99300279888044785</v>
       </c>
-      <c r="S31" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>19</v>
       </c>
       <c r="B32" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C32" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E32" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F32" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="G32" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="H32" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="I32" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="J32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L32" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="M32">
         <v>6</v>
@@ -3752,10 +3766,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P32" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="Q32">
         <v>2.399040383846461E-3</v>
@@ -3763,40 +3777,40 @@
       <c r="R32">
         <v>0.99760095961615358</v>
       </c>
-      <c r="S32" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>19</v>
       </c>
       <c r="B33" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C33" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="D33" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E33" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F33" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="G33" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="H33" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="I33" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="L33" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="M33">
         <v>7</v>
@@ -3805,10 +3819,10 @@
         <v>10.301042495611521</v>
       </c>
       <c r="O33" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P33" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="Q33">
         <v>1.9992003198720509E-4</v>
@@ -3816,8 +3830,8 @@
       <c r="R33">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S33" t="b">
-        <v>0</v>
+      <c r="S33" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
@@ -3825,87 +3839,87 @@
         <v>19</v>
       </c>
       <c r="B34" t="s">
-        <v>284</v>
+        <v>234</v>
       </c>
       <c r="C34" t="s">
-        <v>285</v>
+        <v>235</v>
       </c>
       <c r="D34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E34" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F34" t="s">
-        <v>286</v>
+        <v>236</v>
       </c>
       <c r="G34" t="s">
-        <v>287</v>
+        <v>237</v>
       </c>
       <c r="H34" t="s">
-        <v>288</v>
+        <v>238</v>
       </c>
       <c r="I34" t="s">
-        <v>289</v>
-      </c>
-      <c r="K34" t="s">
-        <v>290</v>
+        <v>239</v>
+      </c>
+      <c r="J34" t="s">
+        <v>45</v>
       </c>
       <c r="L34" t="s">
-        <v>291</v>
+        <v>240</v>
       </c>
       <c r="M34">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N34">
-        <v>2.9999999828690118</v>
+        <v>7.9999999584056276</v>
       </c>
       <c r="O34" t="s">
-        <v>166</v>
+        <v>241</v>
       </c>
       <c r="P34" t="s">
-        <v>166</v>
+        <v>242</v>
       </c>
       <c r="Q34">
-        <v>0.79148340663734507</v>
+        <v>0.22491003598560569</v>
       </c>
       <c r="R34">
-        <v>0.20851659336265491</v>
-      </c>
-      <c r="S34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.77508996401439423</v>
+      </c>
+      <c r="S34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B35" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C35" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D35" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F35" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="G35" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="H35" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="I35" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="L35" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="M35">
         <v>3</v>
@@ -3914,10 +3928,10 @@
         <v>4.1585113396254796</v>
       </c>
       <c r="O35" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="P35" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="Q35">
         <v>5.9976009596161535E-4</v>
@@ -3925,8 +3939,8 @@
       <c r="R35">
         <v>0.99940023990403837</v>
       </c>
-      <c r="S35" t="b">
-        <v>0</v>
+      <c r="S35" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
@@ -3934,63 +3948,66 @@
         <v>19</v>
       </c>
       <c r="B36" t="s">
-        <v>292</v>
+        <v>259</v>
       </c>
       <c r="C36" t="s">
-        <v>301</v>
+        <v>260</v>
       </c>
       <c r="D36" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E36" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F36" t="s">
-        <v>302</v>
+        <v>261</v>
       </c>
       <c r="G36" t="s">
-        <v>303</v>
+        <v>262</v>
       </c>
       <c r="H36" t="s">
-        <v>304</v>
+        <v>263</v>
       </c>
       <c r="I36" t="s">
-        <v>305</v>
+        <v>264</v>
+      </c>
+      <c r="J36" t="s">
+        <v>45</v>
       </c>
       <c r="L36" t="s">
-        <v>306</v>
+        <v>265</v>
       </c>
       <c r="M36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N36">
-        <v>3.9999999792028138</v>
+        <v>7.9999999584056276</v>
       </c>
       <c r="O36" t="s">
-        <v>307</v>
+        <v>142</v>
       </c>
       <c r="P36" t="s">
-        <v>307</v>
+        <v>143</v>
       </c>
       <c r="Q36">
-        <v>0.1367453018792483</v>
+        <v>0.1273490603758497</v>
       </c>
       <c r="R36">
-        <v>0.86325469812075173</v>
-      </c>
-      <c r="S36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.8726509396241503</v>
+      </c>
+      <c r="S36" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>19</v>
       </c>
       <c r="B37" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C37" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -3999,22 +4016,22 @@
         <v>23</v>
       </c>
       <c r="F37" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="G37" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="H37" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="I37" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="J37" t="s">
         <v>28</v>
       </c>
       <c r="L37" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="M37">
         <v>4</v>
@@ -4023,10 +4040,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q37">
         <v>2.1991203518592559E-2</v>
@@ -4034,40 +4051,40 @@
       <c r="R37">
         <v>0.97800879648140748</v>
       </c>
-      <c r="S37" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S37" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C38" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="D38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E38" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F38" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="G38" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="H38" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="I38" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="L38" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="M38">
         <v>3</v>
@@ -4076,10 +4093,10 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O38" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="P38" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="Q38">
         <v>4.7980807676929228E-3</v>
@@ -4087,19 +4104,19 @@
       <c r="R38">
         <v>0.99520191923230705</v>
       </c>
-      <c r="S38" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S38" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C39" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="D39" t="s">
         <v>22</v>
@@ -4108,19 +4125,19 @@
         <v>23</v>
       </c>
       <c r="F39" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="G39" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="H39" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="I39" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="L39" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="M39">
         <v>4</v>
@@ -4129,10 +4146,10 @@
         <v>5.6959538973702619</v>
       </c>
       <c r="O39" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="P39" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="Q39">
         <v>1.9992003198720509E-4</v>
@@ -4140,40 +4157,40 @@
       <c r="R39">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S39" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S39" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>19</v>
       </c>
       <c r="B40" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C40" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D40" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E40" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F40" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="G40" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="H40" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="I40" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="L40" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="M40">
         <v>3</v>
@@ -4182,10 +4199,10 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="P40" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="Q40">
         <v>1.399440223910436E-3</v>
@@ -4193,40 +4210,40 @@
       <c r="R40">
         <v>0.99860055977608952</v>
       </c>
-      <c r="S40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S40" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B41" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C41" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E41" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F41" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="G41" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="H41" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="I41" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L41" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="M41">
         <v>4</v>
@@ -4235,10 +4252,10 @@
         <v>6.8459456886708931</v>
       </c>
       <c r="O41" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P41" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Q41">
         <v>1.7992802878848461E-3</v>
@@ -4246,19 +4263,19 @@
       <c r="R41">
         <v>0.9982007197121151</v>
       </c>
-      <c r="S41" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C42" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="D42" t="s">
         <v>22</v>
@@ -4267,22 +4284,22 @@
         <v>23</v>
       </c>
       <c r="F42" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="G42" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="H42" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="I42" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="J42" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="L42" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="M42">
         <v>5</v>
@@ -4291,10 +4308,10 @@
         <v>9.5533716887630291</v>
       </c>
       <c r="O42" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="P42" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="Q42">
         <v>1.9992003198720512E-3</v>
@@ -4302,43 +4319,43 @@
       <c r="R42">
         <v>0.998000799680128</v>
       </c>
-      <c r="S42" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B43" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="C43" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E43" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F43" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G43" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="H43" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="I43" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="J43" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="L43" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="M43">
         <v>3</v>
@@ -4347,10 +4364,10 @@
         <v>5.4973774838217766</v>
       </c>
       <c r="O43" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="P43" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="Q43">
         <v>6.797281087564974E-3</v>
@@ -4358,19 +4375,19 @@
       <c r="R43">
         <v>0.99320271891243506</v>
       </c>
-      <c r="S43" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S43" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>19</v>
       </c>
       <c r="B44" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C44" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D44" t="s">
         <v>22</v>
@@ -4379,19 +4396,19 @@
         <v>23</v>
       </c>
       <c r="F44" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="G44" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="H44" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="I44" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="L44" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="M44">
         <v>4</v>
@@ -4400,10 +4417,10 @@
         <v>7.4229728235382604</v>
       </c>
       <c r="O44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q44">
         <v>3.9984006397441018E-4</v>
@@ -4411,16 +4428,16 @@
       <c r="R44">
         <v>0.99960015993602558</v>
       </c>
-      <c r="S44" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>19</v>
       </c>
       <c r="B45" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C45" t="s">
         <v>21</v>
@@ -4432,22 +4449,22 @@
         <v>23</v>
       </c>
       <c r="F45" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="G45" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="H45" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="I45" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="J45" t="s">
         <v>28</v>
       </c>
       <c r="L45" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="M45">
         <v>4</v>
@@ -4456,10 +4473,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O45" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P45" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q45">
         <v>9.9960015993602559E-4</v>
@@ -4467,19 +4484,19 @@
       <c r="R45">
         <v>0.99900039984006395</v>
       </c>
-      <c r="S45" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S45" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>19</v>
       </c>
       <c r="B46" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C46" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D46" t="s">
         <v>22</v>
@@ -4488,22 +4505,22 @@
         <v>23</v>
       </c>
       <c r="F46" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="G46" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="H46" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="I46" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="J46" t="s">
         <v>28</v>
       </c>
       <c r="L46" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="M46">
         <v>4</v>
@@ -4512,10 +4529,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O46" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P46" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q46">
         <v>4.1983206717313079E-3</v>
@@ -4523,8 +4540,8 @@
       <c r="R46">
         <v>0.99580167932826869</v>
       </c>
-      <c r="S46" t="b">
-        <v>0</v>
+      <c r="S46" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
@@ -4532,69 +4549,63 @@
         <v>19</v>
       </c>
       <c r="B47" t="s">
-        <v>373</v>
+        <v>296</v>
       </c>
       <c r="C47" t="s">
-        <v>31</v>
+        <v>305</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F47" t="s">
-        <v>374</v>
+        <v>306</v>
       </c>
       <c r="G47" t="s">
-        <v>375</v>
+        <v>307</v>
       </c>
       <c r="H47" t="s">
-        <v>376</v>
+        <v>308</v>
       </c>
       <c r="I47" t="s">
-        <v>377</v>
-      </c>
-      <c r="J47" t="s">
-        <v>28</v>
-      </c>
-      <c r="K47" t="s">
-        <v>378</v>
+        <v>309</v>
       </c>
       <c r="L47" t="s">
-        <v>379</v>
+        <v>310</v>
       </c>
       <c r="M47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N47">
-        <v>4.9999999694042216</v>
+        <v>3.9999999792028138</v>
       </c>
       <c r="O47" t="s">
-        <v>380</v>
+        <v>311</v>
       </c>
       <c r="P47" t="s">
-        <v>381</v>
+        <v>311</v>
       </c>
       <c r="Q47">
-        <v>2.119152339064374E-2</v>
+        <v>0.1367453018792483</v>
       </c>
       <c r="R47">
-        <v>0.97880847660935622</v>
-      </c>
-      <c r="S47" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.86325469812075173</v>
+      </c>
+      <c r="S47" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B48" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="C48" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D48" t="s">
         <v>22</v>
@@ -4603,16 +4614,16 @@
         <v>23</v>
       </c>
       <c r="F48" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="G48" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="H48" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="I48" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="L48" t="s">
         <v>29</v>
@@ -4624,10 +4635,10 @@
         <v>3.4858813438095071</v>
       </c>
       <c r="O48" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="P48" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="Q48">
         <v>1.5993602558976409E-3</v>
@@ -4635,19 +4646,19 @@
       <c r="R48">
         <v>0.99840063974410231</v>
       </c>
-      <c r="S48" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S48" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B49" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C49" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -4656,19 +4667,19 @@
         <v>23</v>
       </c>
       <c r="F49" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="G49" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="H49" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="I49" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="L49" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="M49">
         <v>5</v>
@@ -4677,10 +4688,10 @@
         <v>5.9459063103987697</v>
       </c>
       <c r="O49" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="P49" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="Q49">
         <v>1.9992003198720509E-4</v>
@@ -4688,19 +4699,19 @@
       <c r="R49">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S49" t="b">
-        <v>0</v>
+      <c r="S49" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B50" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="C50" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="D50" t="s">
         <v>22</v>
@@ -4709,19 +4720,19 @@
         <v>23</v>
       </c>
       <c r="F50" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="G50" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="H50" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="I50" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="L50" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="M50">
         <v>2</v>
@@ -4730,10 +4741,10 @@
         <v>3.3753069124198758</v>
       </c>
       <c r="O50" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="P50" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="Q50">
         <v>0.150139944022391</v>
@@ -4741,19 +4752,19 @@
       <c r="R50">
         <v>0.84986005597760894</v>
       </c>
-      <c r="S50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S50" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B51" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="C51" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="D51" t="s">
         <v>22</v>
@@ -4762,19 +4773,19 @@
         <v>23</v>
       </c>
       <c r="F51" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="G51" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="H51" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="I51" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="L51" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="M51">
         <v>6</v>
@@ -4783,10 +4794,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O51" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="P51" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="Q51">
         <v>2.1991203518592559E-3</v>
@@ -4794,19 +4805,19 @@
       <c r="R51">
         <v>0.99780087964814079</v>
       </c>
-      <c r="S51" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S51" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>19</v>
       </c>
       <c r="B52" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C52" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D52" t="s">
         <v>22</v>
@@ -4815,19 +4826,19 @@
         <v>23</v>
       </c>
       <c r="F52" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="G52" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="H52" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="I52" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="L52" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="M52">
         <v>5</v>
@@ -4836,10 +4847,10 @@
         <v>7.9386539795722832</v>
       </c>
       <c r="O52" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="P52" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q52">
         <v>3.9984006397441024E-3</v>
@@ -4847,40 +4858,40 @@
       <c r="R52">
         <v>0.9960015993602559</v>
       </c>
-      <c r="S52" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S52" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>19</v>
       </c>
       <c r="B53" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="C53" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="D53" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E53" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F53" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="G53" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="H53" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="I53" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="L53" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="M53">
         <v>5</v>
@@ -4889,10 +4900,10 @@
         <v>7.9300411159301323</v>
       </c>
       <c r="O53" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="P53" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Q53">
         <v>1.9992003198720509E-4</v>
@@ -4900,40 +4911,40 @@
       <c r="R53">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S53" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S53" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="C54" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="D54" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E54" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F54" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="G54" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="H54" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="I54" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="L54" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="M54">
         <v>4</v>
@@ -4942,10 +4953,10 @@
         <v>7.9999999584056276</v>
       </c>
       <c r="O54" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="P54" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Q54">
         <v>1.1995201919232309E-3</v>
@@ -4953,40 +4964,40 @@
       <c r="R54">
         <v>0.99880047980807674</v>
       </c>
-      <c r="S54" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S54" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B55" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="C55" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="D55" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E55" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F55" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G55" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="H55" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="I55" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="L55" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="M55">
         <v>2</v>
@@ -4995,10 +5006,10 @@
         <v>3.9999999792028138</v>
       </c>
       <c r="O55" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="P55" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="Q55">
         <v>3.5385845661735298E-2</v>
@@ -5006,40 +5017,40 @@
       <c r="R55">
         <v>0.9646141543382647</v>
       </c>
-      <c r="S55" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S55" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>19</v>
       </c>
       <c r="B56" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="C56" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="D56" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E56" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F56" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="G56" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="H56" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="I56" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="L56" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="M56">
         <v>4</v>
@@ -5048,10 +5059,10 @@
         <v>7.5310043681227494</v>
       </c>
       <c r="O56" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P56" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="Q56">
         <v>1.9992003198720509E-4</v>
@@ -5059,40 +5070,40 @@
       <c r="R56">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S56" t="b">
-        <v>0</v>
+      <c r="S56" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B57" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C57" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="D57" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E57" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F57" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="G57" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="H57" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="I57" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="L57" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M57">
         <v>3</v>
@@ -5101,10 +5112,10 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O57" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P57" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q57">
         <v>0.57157137145141945</v>
@@ -5112,40 +5123,40 @@
       <c r="R57">
         <v>0.42842862854858049</v>
       </c>
-      <c r="S57" t="b">
-        <v>0</v>
+      <c r="S57" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B58" t="s">
-        <v>452</v>
+        <v>521</v>
       </c>
       <c r="C58" t="s">
-        <v>447</v>
+        <v>510</v>
       </c>
       <c r="D58" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E58" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F58" t="s">
-        <v>453</v>
+        <v>522</v>
       </c>
       <c r="G58" t="s">
-        <v>454</v>
+        <v>523</v>
       </c>
       <c r="H58" t="s">
-        <v>455</v>
+        <v>524</v>
       </c>
       <c r="I58" t="s">
-        <v>456</v>
+        <v>525</v>
       </c>
       <c r="L58" t="s">
-        <v>457</v>
+        <v>526</v>
       </c>
       <c r="M58">
         <v>3</v>
@@ -5154,72 +5165,75 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O58" t="s">
-        <v>458</v>
+        <v>527</v>
       </c>
       <c r="P58" t="s">
-        <v>458</v>
+        <v>528</v>
       </c>
       <c r="Q58">
-        <v>0.59836065573770492</v>
+        <v>0.99480207916833263</v>
       </c>
       <c r="R58">
-        <v>0.40163934426229508</v>
-      </c>
-      <c r="S58" t="b">
-        <v>1</v>
+        <v>5.1979208316673686E-3</v>
+      </c>
+      <c r="S58" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="B59" t="s">
-        <v>459</v>
+        <v>199</v>
       </c>
       <c r="C59" t="s">
-        <v>447</v>
+        <v>200</v>
       </c>
       <c r="D59" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E59" t="s">
         <v>23</v>
       </c>
       <c r="F59" t="s">
-        <v>460</v>
+        <v>201</v>
       </c>
       <c r="G59" t="s">
-        <v>461</v>
+        <v>202</v>
       </c>
       <c r="H59" t="s">
-        <v>462</v>
+        <v>203</v>
       </c>
       <c r="I59" t="s">
-        <v>463</v>
+        <v>204</v>
+      </c>
+      <c r="J59" t="s">
+        <v>205</v>
       </c>
       <c r="L59" t="s">
-        <v>464</v>
+        <v>206</v>
       </c>
       <c r="M59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N59">
-        <v>1.587351419017982</v>
+        <v>3.422972844335447</v>
       </c>
       <c r="O59" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
       <c r="P59" t="s">
-        <v>86</v>
+        <v>207</v>
       </c>
       <c r="Q59">
-        <v>0.18412634946021589</v>
+        <v>0.1239504198320672</v>
       </c>
       <c r="R59">
-        <v>0.81587365053978411</v>
-      </c>
-      <c r="S59" t="b">
-        <v>1</v>
+        <v>0.87604958016793288</v>
+      </c>
+      <c r="S59" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.2">
@@ -5227,87 +5241,87 @@
         <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>465</v>
+        <v>288</v>
       </c>
       <c r="C60" t="s">
-        <v>466</v>
+        <v>289</v>
       </c>
       <c r="D60" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E60" t="s">
         <v>23</v>
       </c>
       <c r="F60" t="s">
-        <v>467</v>
+        <v>290</v>
       </c>
       <c r="G60" t="s">
-        <v>468</v>
+        <v>291</v>
       </c>
       <c r="H60" t="s">
-        <v>469</v>
+        <v>292</v>
       </c>
       <c r="I60" t="s">
-        <v>470</v>
-      </c>
-      <c r="J60" t="s">
-        <v>44</v>
+        <v>293</v>
+      </c>
+      <c r="K60" t="s">
+        <v>294</v>
       </c>
       <c r="L60" t="s">
-        <v>471</v>
+        <v>295</v>
       </c>
       <c r="M60">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N60">
-        <v>11.99999993760844</v>
+        <v>2.9999999828690118</v>
       </c>
       <c r="O60" t="s">
-        <v>472</v>
+        <v>169</v>
       </c>
       <c r="P60" t="s">
-        <v>472</v>
+        <v>169</v>
       </c>
       <c r="Q60">
-        <v>3.7984806077568968E-3</v>
+        <v>0.79148340663734507</v>
       </c>
       <c r="R60">
-        <v>0.99620151939224311</v>
-      </c>
-      <c r="S60" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
+        <v>0.20851659336265491</v>
+      </c>
+      <c r="S60" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B61" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C61" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="D61" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E61" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F61" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="G61" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="H61" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="I61" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="L61" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="M61">
         <v>6</v>
@@ -5316,10 +5330,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O61" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="P61" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="Q61">
         <v>1.239504198320672E-2</v>
@@ -5327,40 +5341,40 @@
       <c r="R61">
         <v>0.98760495801679327</v>
       </c>
-      <c r="S61" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S61" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B62" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C62" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="D62" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E62" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F62" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="G62" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="H62" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="I62" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="L62" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="M62">
         <v>3</v>
@@ -5369,10 +5383,10 @@
         <v>4.1773810828327207</v>
       </c>
       <c r="O62" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P62" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q62">
         <v>7.9968012794882047E-4</v>
@@ -5380,43 +5394,43 @@
       <c r="R62">
         <v>0.99920031987205116</v>
       </c>
-      <c r="S62" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S62" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>19</v>
       </c>
       <c r="B63" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="C63" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="D63" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E63" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F63" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="G63" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="H63" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="I63" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="J63" t="s">
         <v>28</v>
       </c>
       <c r="L63" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="M63">
         <v>6</v>
@@ -5425,10 +5439,10 @@
         <v>11.99999993760844</v>
       </c>
       <c r="O63" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="P63" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="Q63">
         <v>9.9960015993602559E-4</v>
@@ -5436,19 +5450,19 @@
       <c r="R63">
         <v>0.99900039984006395</v>
       </c>
-      <c r="S63" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S63" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B64" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C64" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="D64" t="s">
         <v>22</v>
@@ -5457,22 +5471,22 @@
         <v>23</v>
       </c>
       <c r="F64" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="G64" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="H64" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="I64" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="J64" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="L64" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="M64">
         <v>3</v>
@@ -5481,10 +5495,10 @@
         <v>2.7321635570580471</v>
       </c>
       <c r="O64" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="P64" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="Q64">
         <v>2.4390243902439029E-2</v>
@@ -5492,40 +5506,40 @@
       <c r="R64">
         <v>0.97560975609756095</v>
       </c>
-      <c r="S64" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S64" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B65" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C65" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="D65" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E65" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F65" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="G65" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="H65" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="I65" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="L65" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="M65">
         <v>4</v>
@@ -5534,10 +5548,10 @@
         <v>5.6354226577422848</v>
       </c>
       <c r="O65" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="P65" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Q65">
         <v>1.9992003198720509E-4</v>
@@ -5545,19 +5559,19 @@
       <c r="R65">
         <v>0.99980007996801279</v>
       </c>
-      <c r="S65" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="S65" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B66" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="C66" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="D66" t="s">
         <v>22</v>
@@ -5566,19 +5580,19 @@
         <v>23</v>
       </c>
       <c r="F66" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="G66" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="H66" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="I66" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="J66" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="L66" t="s">
         <v>29</v>
@@ -5590,10 +5604,10 @@
         <v>4.7472047391684882</v>
       </c>
       <c r="O66" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="P66" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="Q66">
         <v>8.7964814074370252E-3</v>
@@ -5601,40 +5615,40 @@
       <c r="R66">
         <v>0.99120351859256295</v>
       </c>
-      <c r="S66" t="b">
-        <v>0</v>
+      <c r="S66" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B67" t="s">
-        <v>517</v>
+        <v>456</v>
       </c>
       <c r="C67" t="s">
-        <v>506</v>
+        <v>451</v>
       </c>
       <c r="D67" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E67" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F67" t="s">
-        <v>518</v>
+        <v>457</v>
       </c>
       <c r="G67" t="s">
-        <v>519</v>
+        <v>458</v>
       </c>
       <c r="H67" t="s">
-        <v>520</v>
+        <v>459</v>
       </c>
       <c r="I67" t="s">
-        <v>521</v>
+        <v>460</v>
       </c>
       <c r="L67" t="s">
-        <v>522</v>
+        <v>461</v>
       </c>
       <c r="M67">
         <v>3</v>
@@ -5643,104 +5657,104 @@
         <v>5.9999999688042216</v>
       </c>
       <c r="O67" t="s">
-        <v>523</v>
+        <v>462</v>
       </c>
       <c r="P67" t="s">
-        <v>524</v>
+        <v>462</v>
       </c>
       <c r="Q67">
-        <v>0.99480207916833263</v>
+        <v>0.59836065573770492</v>
       </c>
       <c r="R67">
-        <v>5.1979208316673686E-3</v>
-      </c>
-      <c r="S67" t="b">
-        <v>0</v>
+        <v>0.40163934426229508</v>
+      </c>
+      <c r="S67" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="B68" t="s">
-        <v>517</v>
+        <v>463</v>
       </c>
       <c r="C68" t="s">
-        <v>525</v>
+        <v>451</v>
       </c>
       <c r="D68" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E68" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F68" t="s">
-        <v>526</v>
+        <v>464</v>
       </c>
       <c r="G68" t="s">
-        <v>527</v>
+        <v>465</v>
       </c>
       <c r="H68" t="s">
-        <v>528</v>
+        <v>466</v>
       </c>
       <c r="I68" t="s">
-        <v>529</v>
+        <v>467</v>
       </c>
       <c r="L68" t="s">
-        <v>530</v>
+        <v>468</v>
       </c>
       <c r="M68">
         <v>3</v>
       </c>
       <c r="N68">
-        <v>3.2715463687802688</v>
+        <v>1.587351419017982</v>
       </c>
       <c r="O68" t="s">
-        <v>531</v>
+        <v>233</v>
       </c>
       <c r="P68" t="s">
-        <v>532</v>
+        <v>88</v>
       </c>
       <c r="Q68">
-        <v>1.9192323070771691E-2</v>
+        <v>0.18412634946021589</v>
       </c>
       <c r="R68">
-        <v>0.98080767692922832</v>
-      </c>
-      <c r="S68" t="b">
-        <v>1</v>
+        <v>0.81587365053978411</v>
+      </c>
+      <c r="S68" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B69" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="C69" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="D69" t="s">
         <v>22</v>
       </c>
       <c r="E69" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F69" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="G69" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="H69" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="I69" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="L69" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="M69">
         <v>2</v>
@@ -5749,10 +5763,10 @@
         <v>3.9999999792028138</v>
       </c>
       <c r="O69" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="P69" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="Q69">
         <v>0.72371051579368251</v>
@@ -5760,11 +5774,23 @@
       <c r="R69">
         <v>0.27628948420631749</v>
       </c>
-      <c r="S69" t="b">
-        <v>1</v>
+      <c r="S69" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S69" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="18">
+      <filters>
+        <filter val="Strong disagree"/>
+        <filter val="Weak agree"/>
+        <filter val="Weak disagree"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S69">
+      <sortCondition ref="S1:S69"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>